<commit_message>
Rewrite case notes and test records for clearer reading
</commit_message>
<xml_diff>
--- a/balance/coin-survivor-balance.xlsx
+++ b/balance/coin-survivor-balance.xlsx
@@ -1147,7 +1147,7 @@
     </x:row>
     <x:row r="2" ht="50" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>114G에서 상품 네 개(40G)를 사면 74G가 남아 100G 확장을 선택할 수 없었습니다. 구매와 확장을 함께 선택할 여유를 주는 방향을 검토했습니다.</x:v>
+        <x:v>114G로 상품 네 개(40G)를 사면 74G가 남아 100G 확장을 할 수 없었습니다. 구매와 확장을 함께 할 수 있도록 비용을 검토했습니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1172,13 +1172,13 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="15" t="str">
-        <x:v>축</x:v>
+        <x:v>항목</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
         <x:v>목표</x:v>
       </x:c>
       <x:c r="C5" s="15" t="str">
-        <x:v>금지선</x:v>
+        <x:v>피할 상황</x:v>
       </x:c>
       <x:c r="D5" s="15" t="str">
         <x:v>판정 근거</x:v>
@@ -1203,10 +1203,10 @@
         <x:v>생존 경제</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>상점은 유료지만 진입 후 40G 이상 보존</x:v>
+        <x:v>진입비를 낸 뒤에도 40G 이상 남기기</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>진입비 0G / 아이템을 못 사는 악순환</x:v>
+        <x:v>무료 진입 / 구매할 골드 부족</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
         <x:v>성장 곡선 + 실제 상점 전후 골드</x:v>
@@ -1231,13 +1231,13 @@
         <x:v>성장 체감</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>몸집은 커지되 화면과 판정이 같은 상태</x:v>
+        <x:v>몸집·화면·충돌 판정의 성장 단계 일치</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
         <x:v>상점 정지 중 외형·판정 불일치</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>성장·카메라 상태 전이 체크</x:v>
+        <x:v>성장·카메라 변경 시점 확인</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1295,7 +1295,7 @@
         <x:v>0보다 크고 완만한 증가</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>정적 반영</x:v>
+        <x:v>코드 반영</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
         <x:v>Play Mode에서 상점 1~5회 잔여 골드 기록</x:v>
@@ -1312,7 +1312,7 @@
         <x:v>이전 2.5 대비 20% 하향</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>정적 반영</x:v>
+        <x:v>코드 반영</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
         <x:v>패시브 없이 체감 확인</x:v>
@@ -1329,7 +1329,7 @@
         <x:v>성장 단계 6.0/6.6/7.32/8.1</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>정적 반영</x:v>
+        <x:v>코드 반영</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
         <x:v>상점·피격 전후 프레이밍 확인</x:v>
@@ -1346,7 +1346,7 @@
         <x:v>스냅샷 총 6 이하</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>정적 반영</x:v>
+        <x:v>코드 반영</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
         <x:v>화면 밖 피해율과 투사체 가독성 확인</x:v>
@@ -1388,7 +1388,7 @@
         <x:v>구간</x:v>
       </x:c>
       <x:c r="B22" s="15" t="str">
-        <x:v>플레이 감정</x:v>
+        <x:v>플레이 목표</x:v>
       </x:c>
       <x:c r="C22" s="15" t="str">
         <x:v>근거리 압력</x:v>
@@ -1481,7 +1481,7 @@
         <x:v>12분</x:v>
       </x:c>
       <x:c r="G25" s="12" t="str">
-        <x:v>경제가 선택을 봉쇄</x:v>
+        <x:v>구매·확장 불가</x:v>
       </x:c>
       <x:c r="H25" s="12" t="str">
         <x:v>드랍/아이템/확장비</x:v>
@@ -1558,7 +1558,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>상점은 timeScale 0이므로 성장 갱신을 잠그고, 닫힐 때 골드 기준 상태를 한 번에 재적용합니다.</x:v>
+        <x:v>상점에서는 timeScale이 0인 동안 성장을 고정하고 닫을 때 보유 골드에 맞춰 외형·판정·카메라를 갱신합니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1747,7 +1747,7 @@
     <x:row r="10"/>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="8" t="str">
-        <x:v>필수 상태 전이</x:v>
+        <x:v>확인할 상태 변화</x:v>
       </x:c>
       <x:c r="B11" s="8"/>
       <x:c r="C11" s="8"/>
@@ -1816,7 +1816,7 @@
         <x:v>고정</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>여러 골드 변화에도 단일 상태</x:v>
+        <x:v>골드가 바뀌어도 상태 고정</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -1929,7 +1929,7 @@
     </x:row>
     <x:row r="2" ht="36" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>노란 칸에 실제 측정값을 입력합니다. 판정에 필요한 원거리 적 수, 화면 안·밖 피해, FPS, 1% low, 오류 수가 모두 숫자여야 판정합니다.</x:v>
+        <x:v>노란 칸에 실측값을 입력합니다. 원거리 적 수·화면 안팎 피해·FPS·1% low·오류 수가 모두 숫자여야 판정합니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -2183,7 +2183,7 @@
     <x:row r="15"/>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="8" t="str">
-        <x:v>회귀 체크리스트</x:v>
+        <x:v>수정 후 함께 확인할 기능</x:v>
       </x:c>
       <x:c r="B16" s="8"/>
       <x:c r="C16" s="8"/>
@@ -2224,7 +2224,7 @@
         <x:v>Start 업그레이드 한글</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>ㅁㅁㅁ 없음</x:v>
+        <x:v>한글이 네모로 깨지지 않음</x:v>
       </x:c>
       <x:c r="D18" s="16" t="str">
         <x:v>미측정</x:v>
@@ -2239,7 +2239,7 @@
         <x:v>상점 진입/종료 반복</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>pause owner 누수·중복 이자 없음</x:v>
+        <x:v>일시정지 해제·이자 1회 지급</x:v>
       </x:c>
       <x:c r="D19" s="16" t="str">
         <x:v>미측정</x:v>
@@ -2329,7 +2329,7 @@
         <x:v>저장/불러오기</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>빈/구버전 슬롯 안전, 플레이타임 증가</x:v>
+        <x:v>빈 슬롯·구버전 슬롯 처리 / 플레이시간 증가</x:v>
       </x:c>
       <x:c r="D25" s="16" t="str">
         <x:v>미측정</x:v>
@@ -2365,7 +2365,7 @@
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>데이터 품질·추적성</x:v>
+        <x:v>출처와 확인 방법</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -2377,7 +2377,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정적 사실, 계산식, Play Mode 실측, 설계 목표를 구분합니다.</x:v>
+        <x:v>코드에서 읽은 값·수식 계산·플레이 측정·설계 목표를 나눠 기록합니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -2587,7 +2587,7 @@
         <x:v>맵 이탈·복귀</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>정적 재현 불가</x:v>
+        <x:v>코드 분석만으로 확인 어려움</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
         <x:v>플레이 확인</x:v>
@@ -2612,7 +2612,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="15" t="str">
-        <x:v>검증 층</x:v>
+        <x:v>확인 방법</x:v>
       </x:c>
       <x:c r="B15" s="15" t="str">
         <x:v>확인한 내용</x:v>
@@ -2690,7 +2690,7 @@
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>현재 코드 기준</x:v>
+        <x:v>기준값과 출처</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -2700,7 +2700,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>2026-07-16 정적 반영값. 노란색은 Play Mode에서 입력할 값입니다.</x:v>
+        <x:v>2026-07-16 코드·데이터 기준. 노란 칸에는 실제 플레이 측정값을 입력합니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -3091,7 +3091,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>진입은 무료가 아니며, 진행 조건과 생존 골드 조건을 동시에 만족해야 합니다.</x:v>
+        <x:v>상점은 누적 획득 목표를 채우고 진입비를 낸 뒤에도 생존 골드가 남아야 열립니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -3674,7 +3674,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>baseCount는 초당 생성량이 아니라 유지 목표 수입니다. 근거리만 증량하고 원거리 상한은 유지했습니다.</x:v>
+        <x:v>baseCount는 유지할 적 수입니다. 초당 생성량이 아닙니다. 근거리 목표를 늘리고 원거리 상한은 유지했습니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -4612,7 +4612,7 @@
     <x:row r="21"/>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="20" t="str">
-        <x:v>스냅샷 목표 수</x:v>
+        <x:v>시각별 적 유지 목표</x:v>
       </x:c>
       <x:c r="B22" s="20"/>
       <x:c r="C22" s="20"/>
@@ -4776,7 +4776,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>고밀도에서는 개체 공격력을 낮추고, 보스 체력·보상은 출현 시간에 따라 단조 증가시킵니다.</x:v>
+        <x:v>적이 많아지는 구간은 개체별 공격력을 낮췄습니다. 보스 체력과 보상은 출현 시각에 따라 늘어납니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -4826,7 +4826,7 @@
         <x:v>100G 기준 피격 허용 횟수</x:v>
       </x:c>
       <x:c r="L4" s="15" t="str">
-        <x:v>정적 비고</x:v>
+        <x:v>코드·데이터 비고</x:v>
       </x:c>
       <x:c r="N4" t="str">
         <x:v>보스</x:v>
@@ -5360,7 +5360,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>골드는 체력·경험치·상점 재화입니다. 셋 중 하나만 최적화하면 게임이 불쾌해집니다.</x:v>
+        <x:v>골드는 체력·경험치·구매 재화에 함께 쓰이므로 소비와 생존을 같이 봅니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -5525,7 +5525,7 @@
     <x:row r="10"/>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="8" t="str">
-        <x:v>경제 안전 규칙</x:v>
+        <x:v>구매·보상 처리 규칙</x:v>
       </x:c>
       <x:c r="B11" s="8"/>
       <x:c r="C11" s="8"/>
@@ -5559,7 +5559,7 @@
         <x:v>누적 진행 충족 AND 현재G-진입비&gt;=40</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>경험치 문턱과 생존 문턱 분리</x:v>
+        <x:v>성장 진행도와 생존 골드 구분</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
         <x:v>반영</x:v>
@@ -5573,7 +5573,7 @@
         <x:v>기존 아이템 합성 우선, 없으면 빈칸</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>빈칸 부족 때문에 합성 기회 차단 금지</x:v>
+        <x:v>빈칸이 없어도 합성 가능한 구매는 허용</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
         <x:v>반영</x:v>
@@ -5587,7 +5587,7 @@
         <x:v>현재G+판매가&lt;=최대G</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>한도 클램프로 아이템만 사라지는 손실 금지</x:v>
+        <x:v>골드 한도로 아이템만 잃는 상황 방지</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
         <x:v>반영</x:v>
@@ -5601,7 +5601,7 @@
         <x:v>모든 후보 배치 실패 시 10 다이아</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>100 다이아 과보상 방지</x:v>
+        <x:v>상자 배치 실패 보상 제한</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
         <x:v>반영</x:v>
@@ -5615,7 +5615,7 @@
         <x:v>상점 true→false 전이당 1회</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>중복 닫기 이벤트로 중복 지급 금지</x:v>
+        <x:v>상점 종료 시 이자 중복 지급 방지</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
         <x:v>반영</x:v>
@@ -5667,7 +5667,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>초반은 싸게 열고 후반 선택은 가파르게 만듭니다. 동일 패시브는 Common 환산 4개가 절대 상한입니다.</x:v>
+        <x:v>초반 확장비는 낮게 두고 후반으로 갈수록 높였습니다. 동일 패시브는 Common 환산 4개까지만 보유할 수 있습니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -5742,7 +5742,7 @@
         <x:v>710</x:v>
       </x:c>
       <x:c r="J5" s="12" t="str">
-        <x:v>초반 선택 허용, 후반 기회비용</x:v>
+        <x:v>초반 확장 부담 완화 / 후반 비용 증가</x:v>
       </x:c>
     </x:row>
     <x:row r="6"/>
@@ -5974,7 +5974,7 @@
         <x:v>최대 판매가</x:v>
       </x:c>
       <x:c r="J17" s="15" t="str">
-        <x:v>선택 압력</x:v>
+        <x:v>배치할 때 볼 점</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -6226,7 +6226,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>패시브는 현재 장착 등급 1개만 적용됩니다. 동일 패시브 구매 한도는 Common 환산 4개입니다.</x:v>
+        <x:v>현재 장착한 등급의 효과 하나만 적용됩니다. 같은 패시브는 Common 환산 4개까지 구매할 수 있습니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -6248,7 +6248,7 @@
         <x:v>한글 역할</x:v>
       </x:c>
       <x:c r="C4" s="15" t="str">
-        <x:v>발동 축</x:v>
+        <x:v>효과</x:v>
       </x:c>
       <x:c r="D4" s="15" t="str">
         <x:v>Common</x:v>
@@ -6454,7 +6454,7 @@
     <x:row r="11"/>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="8" t="str">
-        <x:v>시너지 안전 예산</x:v>
+        <x:v>조합별 상한과 확인 기준</x:v>
       </x:c>
       <x:c r="B12" s="8"/>
       <x:c r="C12" s="8"/>
@@ -6481,7 +6481,7 @@
         <x:v>성능/가독성 위험</x:v>
       </x:c>
       <x:c r="E13" s="15" t="str">
-        <x:v>허용 판정</x:v>
+        <x:v>유지 조건</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
@@ -6584,7 +6584,7 @@
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>무기별 유효 사이클과 Play Mode DPS</x:v>
+        <x:v>무기별 계산값과 실측 DPS</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -6602,7 +6602,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정적 프록시는 비교 보조일 뿐입니다. 최종 DPS는 새 텔레메트리의 10초 실측값으로만 판정합니다.</x:v>
+        <x:v>비교용 계산과 실제 피해량을 나눴습니다. 실전 DPS는 10초 동안 측정한 피해량으로 확인합니다.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -6639,7 +6639,7 @@
         <x:v>지속/반경</x:v>
       </x:c>
       <x:c r="G4" s="15" t="str">
-        <x:v>정적 1대상 프록시</x:v>
+        <x:v>1대상 비교 계산</x:v>
       </x:c>
       <x:c r="H4" s="15" t="str">
         <x:v>유효 사거리</x:v>
@@ -6904,7 +6904,7 @@
         <x:v>실패 의미</x:v>
       </x:c>
       <x:c r="D14" s="15" t="str">
-        <x:v>첫 조정 레버</x:v>
+        <x:v>우선 검토할 항목</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -6943,7 +6943,7 @@
         <x:v>&lt;=25%</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>수치가 DPS로 낭비</x:v>
+        <x:v>남은 체력보다 과도한 피해</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
         <x:v>피해 분산·타깃 선택</x:v>

</xml_diff>